<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.002-02 Nino et le bateau de papier
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.002-02.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.002-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Après la pluie, Nino pose son bateau de papier dans une flaque. Le papier se déchire. Il dit qu'il est triste. Il demande un câlin.</t>
+          <t>Une goutte tape la capuche. Sur le tissu, un éclat de capuche luit. Nino veut le bateau de papier, maintenant. L'eau l'emporte. Le papier se déchire. Poitrine trop vite. Sourire parti. Yeux chauds. Je suis triste. Nino pleure. Papa s'accroupit. Deuxième ruse : le papier se déchire plus loin, le bateau part. Il refuse de foncer. Je veux un câlin. Merci vécu. Un éclat de capuche tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Après la pluie, le parc sent le bois mouillé. Les bancs brillent. L'herbe est lourde. Une feuille collée au banc sèche tout doucement. Ça sent la terre mouillée. Une flaque ronde attend près de l'allée. Maman tient le manteau de Nino. Papa arrive avec un sac, un peu plus loin. Nino, tu as ton bateau de papier ? Oui. Il est dans ma poche. On reste près de l'allée, d'accord ? D'accord, papa. En ce moment, Nino sort le bateau. Le papier est encore bien plié. Un pli au milieu. Deux bouts comme des ailes. Il le pose dans la flaque, tout doucement. L'eau emporte le bateau d'un tout petit coup. Le papier se ramollit. Il se déchire. Mon bateau... Parce que le bateau est parti, Nino sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Nino pleure un peu. Les larmes coulent. Elles sont chaudes. Je m'assois sur le banc. Je t'écoute. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Nino se blottit. Le câlin est chaud. Le manteau sent la pluie. Le papier est mouillé. On le laisse. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Nino. Le câlin aide. Oui. Le câlin aide. La flaque reste là, toute calme. Un oiseau saute près du banc. Tu veux rester contre maman un moment ? Oui, papa.</t>
+          <t>Une goutte tape la capuche de Nino. Elle tape, papa. Tu l'entends, la goutte ? Oui, papa. Le parc, après la pluie, goutte partout. Tu le sens, l'air mouillé ? Oui, maman. Sur le tissu, un éclat de capuche luit. Il brille, maman. Tu le vois, sur le tissu ? Oui, un petit point. La goutte le touche. L'air sent la terre, un peu mouillée. Ça sent l'eau. Tes mains sont froides, Nino ? Un peu, maman. Nino met les mains dans sa poche. Il est là. C'est ton bateau de papier ? Oui, maman. Le papier est un peu froid. Il colle aux doigts. Tu le sors, Nino ? Oui, papa. Le bateau a un pli au milieu. Deux bouts, comme des ailes. Il est petit, Nino ? Oui, tout petit. Une flaque ronde attend près de l'allée. Elle est ronde ! Tu la vois, la flaque ? Oui, papa. L'herbe est lourde, près de l'eau. Elle colle aux chaussures. Tes chaussures sont mouillées, Nino ? Un peu, maman. En ce moment, Nino avance vers la flaque. Je veux le bateau, maintenant ! Tout de suite ? Oui, papa. Il pose le bateau sur l'eau. L'eau emporte le bateau d'un petit coup. Le papier se ramollit. Le papier se déchire. Mon bateau ! Nino reste surpris, les mains ouvertes. Sa gorge se serre un peu. Sa poitrine va trop vite. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Nino pleure un peu. Les larmes sont chaudes, sur ses joues. Papa s'accroupit à la même hauteur. Tu vois le bateau, Nino ? Oui, papa. Tes yeux sont chauds, Nino ? Un peu, maman. L'éclat de capuche tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Après la pluie, le parc sent le bois mouillé. Les bancs brillent. L'herbe est lourde. Une feuille collée au banc sèche tout doucement. Ça sent la terre mouillée. Une flaque ronde attend près de l'allée. Maman tient le manteau de Nino. Papa arrive avec un sac, un peu plus loin. Nino, tu as ton bateau de papier ? Oui. Il est dans ma poche. On reste près de l'allée, d'accord ? D'accord, papa. En ce moment, Nino sort le bateau. Le papier est encore bien plié. Un pli au milieu. Deux bouts comme des ailes. Il le pose dans la flaque, tout doucement. L'eau emporte le bateau d'un tout petit coup. Le papier se ramollit. Il se déchire. Mon bateau... Parce que le bateau est parti, Nino sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Tu es triste. C'est permis. Pleurer est permis. Nino pleure un peu. Les larmes coulent. Elles sont chaudes. Je m'assois sur le banc. Je t'écoute. Je veux un câlin. Viens. Un câlin. Maman ouvre les bras. Nino se blottit. Le câlin est chaud. Le manteau sent la pluie. Le papier est mouillé. On le laisse. Tu as dit : je suis triste. Bravo. Tu as demandé un câlin. Pleurer est permis, Nino. Le câlin aide. Oui. Le câlin aide. La flaque reste là, toute calme. Un oiseau saute près du banc. Tu veux rester contre maman un moment ? Oui, papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une goutte tape la capuche de Nino. Elle tape, papa. Tu l'entends, la goutte ? Oui, papa. Le parc, après la pluie, goutte partout. Tu le sens, l'air mouillé ? Oui, maman. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de capuche&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le tissu ? Oui, un petit point. La goutte le touche. L'air sent la terre, un peu mouillée. Ça sent l'eau. Tes mains sont froides, Nino ? Un peu, maman. Nino met les mains dans sa poche. Il est là. C'est ton bateau de papier ? Oui, maman. Le papier est un peu froid. Il colle aux doigts. Tu le sors, Nino ? Oui, papa. Le bateau a un pli au milieu. Deux bouts, comme des ailes. Il est petit, Nino ? Oui, tout petit. Une flaque ronde attend près de l'allée. Elle est ronde ! Tu la vois, la flaque ? Oui, papa. L'herbe est lourde, près de l'eau. Elle colle aux chaussures. Tes chaussures sont mouillées, Nino ? Un peu, maman. En ce moment, Nino avance vers la flaque. Je veux le bateau, maintenant ! Tout de suite ? Oui, papa. Il pose le bateau sur l'eau. L'eau emporte le bateau d'un petit coup. Le papier se ramollit. Le papier se déchire. Mon bateau ! Nino reste surpris, les mains ouvertes. Sa gorge se serre un peu. Sa poitrine va trop vite. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Nino pleure un peu. Les larmes sont chaudes, sur ses joues. Papa s'accroupit à la même hauteur. Tu vois le bateau, Nino ? Oui, papa. Tes yeux sont chauds, Nino ? Un peu, maman. L'éclat de capuche tremble, puis tient.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Nino est au parc avec maman. Il a un bateau en papier. Il le pose dans une flaque. L'eau emporte le bateau. Le papier se déchire. Parce que le bateau est parti, Nino sent sa gorge serrée. Ses yeux deviennent chauds. Une larme tombe. Nino dit : je suis &lt;emphasis&gt;triste&lt;/emphasis&gt;. Maman arrive près de lui. Maman dit : pleurer est permis. Nino pleure un peu. Les larmes coulent. Puis Nino dit : je veux un câlin. Maman ouvre les bras. Nino se blottit. Le câlin est chaud. Papa arrive aussi. Il s'assoit sur le banc. Être triste, c'est permis. Le câlin aide. Nino respire. Maman reste près de lui. [pause]</t>
+          <t>Une goutte tape la capuche de Nino. Elle tape, papa. Tu l'entends, la goutte ? Oui, papa. Le parc, après la pluie, goutte partout. Tu le sens, l'air mouillé ? Oui, maman. Sur le tissu, un &lt;emphasis&gt;éclat de capuche&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le tissu ? Oui, un petit point. La goutte le touche. L'air sent la terre, un peu mouillée. Ça sent l'eau. Tes mains sont froides, Nino ? Un peu, maman. Nino met les mains dans sa poche. Il est là. C'est ton bateau de papier ? Oui, maman. Le papier est un peu froid. Il colle aux doigts. Tu le sors, Nino ? Oui, papa. Le bateau a un pli au milieu. Deux bouts, comme des ailes. Il est petit, Nino ? Oui, tout petit. Une flaque ronde attend près de l'allée. Elle est ronde ! Tu la vois, la flaque ? Oui, papa. L'herbe est lourde, près de l'eau. Elle colle aux chaussures. Tes chaussures sont mouillées, Nino ? Un peu, maman. En ce moment, Nino avance vers la flaque. Je veux le bateau, maintenant ! Tout de suite ? Oui, papa. Il pose le bateau sur l'eau. L'eau emporte le bateau d'un petit coup. Le papier se ramollit. Le papier se déchire. Mon bateau ! Nino reste surpris, les mains ouvertes. Sa gorge se serre un peu. Sa poitrine va trop vite. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Ses épaules tombent un peu. Ses yeux deviennent chauds. Une larme tombe. Je suis triste. Nino pleure un peu. Les larmes sont chaudes, sur ses joues. Papa s'accroupit à la même hauteur. Tu vois le bateau, Nino ? Oui, papa. Tes yeux sont chauds, Nino ? Un peu, maman. L'éclat de capuche tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>éclat de capuche</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,51 +1321,76 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=élan puis tristesse; intensite=2; destinataire=enfant; sous_texte=il_veut_le_bateau_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Après la pluie, le parc sent le bois mouillé.
-narrateur|Les bancs brillent. L'herbe est lourde.
-narrateur|Une feuille collée au banc sèche tout doucement.
-narrateur|Ça sent la terre mouillée.
+          <t>narrateur|Une goutte tape la capuche de Nino.
+enfant-m|Elle tape, papa.
+papa|Tu l'entends, la goutte ?
+enfant-m|Oui, papa.
+narrateur|Le parc, après la pluie, goutte partout.
+maman|Tu le sens, l'air mouillé ?
+enfant-m|Oui, maman.
+narrateur|Sur le tissu, un éclat de capuche luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le tissu ?
+enfant-m|Oui, un petit point.
+papa|La goutte le touche.
+narrateur|L'air sent la terre, un peu mouillée.
+enfant-m|Ça sent l'eau.
+maman|Tes mains sont froides, Nino ?
+enfant-m|Un peu, maman.
+narrateur|Nino met les mains dans sa poche.
+enfant-m|Il est là.
+maman|C'est ton bateau de papier ?
+enfant-m|Oui, maman.
+narrateur|Le papier est un peu froid.
+enfant-m|Il colle aux doigts.
+papa|Tu le sors, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le bateau a un pli au milieu.
+enfant-m|Deux bouts, comme des ailes.
+maman|Il est petit, Nino ?
+enfant-m|Oui, tout petit.
 narrateur|Une flaque ronde attend près de l'allée.
-narrateur|Maman tient le manteau de Nino.
-narrateur|Papa arrive avec un sac, un peu plus loin.
-maman|Nino, tu as ton bateau de papier ?
-enfant-m|Oui. Il est dans ma poche.
-papa|On reste près de l'allée, d'accord ?
-enfant-m|D'accord, papa.
-narrateur|En ce moment, Nino sort le bateau.
-narrateur|Le papier est encore bien plié.
-narrateur|Un pli au milieu. Deux bouts comme des ailes.
-narrateur|Il le pose dans la flaque, tout doucement.
-narrateur|L'eau emporte le bateau d'un tout petit coup.
-narrateur|Le papier se ramollit. Il se déchire.
-enfant-m|Mon bateau...
-narrateur|Parce que le bateau est parti, Nino sent sa gorge serrée.
+enfant-m|Elle est ronde !
+papa|Tu la vois, la flaque ?
+enfant-m|Oui, papa.
+narrateur|L'herbe est lourde, près de l'eau.
+enfant-m|Elle colle aux chaussures.
+maman|Tes chaussures sont mouillées, Nino ?
+enfant-m|Un peu, maman.
+narrateur|En ce moment, Nino avance vers la flaque.
+enfant-m|Je veux le bateau, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Il pose le bateau sur l'eau.
+narrateur|L'eau emporte le bateau d'un petit coup.
+narrateur|Le papier se ramollit.
+narrateur|Le papier se déchire.
+enfant-m|Mon bateau !
+narrateur|Nino reste surpris, les mains ouvertes.
+narrateur|Sa gorge se serre un peu.
+narrateur|Sa poitrine va trop vite.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+narrateur|Ses épaules tombent un peu.
 narrateur|Ses yeux deviennent chauds.
 narrateur|Une larme tombe.
 enfant-m|Je suis triste.
-maman|Tu es triste. C'est permis.
-maman|Pleurer est permis.
 narrateur|Nino pleure un peu.
-narrateur|Les larmes coulent. Elles sont chaudes.
-papa|Je m'assois sur le banc. Je t'écoute.
-enfant-m|Je veux un câlin.
-maman|Viens. Un câlin.
-narrateur|Maman ouvre les bras.
-narrateur|Nino se blottit. Le câlin est chaud.
-narrateur|Le manteau sent la pluie.
-papa|Le papier est mouillé. On le laisse.
-maman|Tu as dit : je suis triste.
-maman|Bravo. Tu as demandé un câlin.
-papa|Pleurer est permis, Nino.
-enfant-m|Le câlin aide.
-maman|Oui. Le câlin aide.
-narrateur|La flaque reste là, toute calme.
-narrateur|Un oiseau saute près du banc.
-papa|Tu veux rester contre maman un moment ?
-enfant-m|Oui, papa.</t>
+narrateur|Les larmes sont chaudes, sur ses joues.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois le bateau, Nino ?
+enfant-m|Oui, papa.
+maman|Tes yeux sont chauds, Nino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de capuche tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1402,12 +1427,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a les yeux chauds. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Nino&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Nino a les yeux chauds. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Nino&lt;/emphasis&gt; a les yeux chauds. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1470,7 +1495,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1481,7 +1506,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1496,34 +1521,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nino</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1538,22 +1567,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_a_les_yeux_chauds_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Nino a les yeux chauds. Que dit-il ?</t>
+          <t>narrateur|Nino a les yeux chauds.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1580,17 +1610,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nino sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Le câlin aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Maman le serre, sans se presser. Le banc est un peu froid sous papa.</t>
+          <t>Nino veut le bateau, tout de suite. Je le prends, maintenant ! Le bateau reste un peu loin, dans l'eau. Les mots se bousculent dans sa bouche. Trop vite. Nino avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Il est mouillé. Tu restes un peu, Nino ? Oui, papa. Papa reste à la même hauteur. Le papier est mou, sous les doigts. Il pique un peu. Nino reprend le bord du papier, sans se presser. Tu le vois, le bateau ? Oui, papa. Il tient, Nino ? Un peu, maman. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la flaque ? Oui. La goutte tape la capuche ? Oui, maman. Un pli du bateau attend sur l'eau. Je le prends. Tu le poses, Nino ? Pas tout de suite. Le papier a une petite déchirure. Il est déchiré. Tes genoux sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nino sèche une larme avec sa manche. Je suis triste. Oui. Et pleurer est permis. Le câlin aide. Bravo. Tu as dit ce que tu sentais. Tu veux encore un câlin ? Encore un peu. Maman le serre, sans se presser. Le banc est un peu froid sous papa.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut le bateau, tout de suite. Je le prends, maintenant ! Le bateau reste un peu loin, dans l'eau. Les mots se bousculent dans sa bouche. Trop vite. Nino avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Il est mouillé. Tu restes un peu, Nino ? Oui, papa. Papa reste à la même hauteur. Le &lt;emphasis level="moderate"&gt;papier&lt;/emphasis&gt; est mou, sous les doigts. Il pique un peu. Nino reprend le bord du papier, sans se presser. Tu le vois, le bateau ? Oui, papa. Il tient, Nino ? Un peu, maman. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la flaque ? Oui. La goutte tape la capuche ? Oui, maman. Un pli du bateau attend sur l'eau. Je le prends. Tu le poses, Nino ? Pas tout de suite. Le papier a une petite déchirure. Il est déchiré. Tes genoux sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Nino a nommé : &lt;emphasis&gt;triste&lt;/emphasis&gt;. Pleurer est permis. Un câlin de maman aide. [pause]</t>
+          <t>Nino veut le bateau, tout de suite. Je le prends, maintenant ! Le bateau reste un peu loin, dans l'eau. Les mots se bousculent dans sa bouche. Trop vite. Nino avance les mains, trop vite. Puis il s'arrête. Il referme la bouche. Personne ne parle. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Il est mouillé. Tu restes un peu, Nino ? Oui, papa. Papa reste à la même hauteur. Le &lt;emphasis&gt;papier&lt;/emphasis&gt; est mou, sous les doigts. Il pique un peu. Nino reprend le bord du papier, sans se presser. Tu le vois, le bateau ? Oui, papa. Il tient, Nino ? Un peu, maman. Le ventre de Nino se desserre. Les épaules se relèvent un peu. On reste près de la flaque ? Oui. La goutte tape la capuche ? Oui, maman. Un pli du bateau attend sur l'eau. Je le prends. Tu le poses, Nino ? Pas tout de suite. Le papier a une petite déchirure. Il est déchiré. Tes genoux sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1648,7 +1678,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1671,7 +1701,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>triste</t>
+          <t>papier</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1685,16 +1715,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1719,20 +1749,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer_sans_leçon; emotion=retenue puis souffle_plus_large; intensite=1; destinataire=enfant; sous_texte=il_s_arrete_le_papier_tient; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nino sèche une larme avec sa manche.
-enfant-m|Je suis triste.
-maman|Oui. Et pleurer est permis.
-maman|Le câlin aide.
-papa|Bravo. Tu as dit ce que tu sentais.
-papa|Tu veux encore un câlin ?
-enfant-m|Encore un peu.
-narrateur|Maman le serre, sans se presser.
-narrateur|Le banc est un peu froid sous papa.</t>
+          <t>narrateur|Nino veut le bateau, tout de suite.
+enfant-m|Je le prends, maintenant !
+narrateur|Le bateau reste un peu loin, dans l'eau.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-m|Trop vite.
+narrateur|Nino avance les mains, trop vite.
+narrateur|Puis il s'arrête.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe la flaque, un instant.
+narrateur|Il écoute le parc, près de l'allée.
+enfant-m|Il est mouillé.
+papa|Tu restes un peu, Nino ?
+enfant-m|Oui, papa.
+narrateur|Papa reste à la même hauteur.
+maman|Le papier est mou, sous les doigts.
+enfant-m|Il pique un peu.
+narrateur|Nino reprend le bord du papier, sans se presser.
+papa|Tu le vois, le bateau ?
+enfant-m|Oui, papa.
+maman|Il tient, Nino ?
+enfant-m|Un peu, maman.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la flaque ?
+enfant-m|Oui.
+maman|La goutte tape la capuche ?
+enfant-m|Oui, maman.
+narrateur|Un pli du bateau attend sur l'eau.
+enfant-m|Je le prends.
+papa|Tu le poses, Nino ?
+enfant-m|Pas tout de suite.
+narrateur|Le papier a une petite déchirure.
+enfant-m|Il est déchiré.
+maman|Tes genoux sont au chaud ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
     </row>
@@ -1759,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino sèche ses joues. Le parc sent encore le bois mouillé. On rentre quand tu es prêt ? Encore le banc. On reste. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent au banc, tout près. La flaque ne bouge plus.</t>
+          <t>Maman pousse un peu l'herbe près de l'eau. L'herbe est un peu froide. Le bateau, maintenant ! Nino approche la main, trop vite. Le papier se déchire, plus loin. Il se déchire ! Le bateau part vers le milieu. Il part ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Sur le tissu, un éclat de capuche luit. Là, sur le tissu. Nino attend, les mains ouvertes. Je veux un câlin. Tu viens, Nino ? Oui, maman. Maman ouvre les bras. Nino se blottit contre le manteau. Merci, Nino. Le manteau sent la pluie, un peu tiède. Il est chaud. Nino pose la joue sur le manteau. Ça sent la pluie. La capuche est mouillée, Nino ? Un peu. Tu vois le point, Nino ? Oui, papa. Le bateau tient, un peu déchiré. On le garde. Une goutte passe sur la capuche. Elle tape. On reste ici, Nino ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino sèche ses joues. Le parc sent encore le bois mouillé. On rentre quand tu es prêt ? Encore le banc. On reste. Tu as bien demandé le câlin. Je suis moins triste. Le câlin est encore là. Ils restent au banc, tout près. La flaque ne bouge plus.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pousse un peu l'herbe près de l'eau. L'herbe est un peu froide. Le bateau, maintenant ! Nino approche la main, trop vite. Le papier se déchire, plus loin. Il se déchire ! Le bateau part vers le milieu. Il part ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Sur le tissu, un &lt;emphasis level="moderate"&gt;éclat de capuche&lt;/emphasis&gt; luit. Là, sur le tissu. Nino attend, les mains ouvertes. Je veux un câlin. Tu viens, Nino ? Oui, maman. Maman ouvre les bras. Nino se blottit contre le manteau. Merci, Nino. Le manteau sent la pluie, un peu tiède. Il est chaud. Nino pose la joue sur le manteau. Ça sent la pluie. La capuche est mouillée, Nino ? Un peu. Tu vois le point, Nino ? Oui, papa. Le bateau tient, un peu déchiré. On le garde. Une goutte passe sur la capuche. Elle tape. On reste ici, Nino ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Nino sèche ses joues. Papa reste au banc. [pause]</t>
+          <t>Maman pousse un peu l'herbe près de l'eau. L'herbe est un peu froide. Le bateau, maintenant ! Nino approche la main, trop vite. Le papier se déchire, plus loin. Il se déchire ! Le bateau part vers le milieu. Il part ! Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe la flaque, un instant. Il écoute le parc, près de l'allée. Sur le tissu, un &lt;emphasis&gt;éclat de capuche&lt;/emphasis&gt; luit. Là, sur le tissu. Nino attend, les mains ouvertes. Je veux un câlin. Tu viens, Nino ? Oui, maman. Maman ouvre les bras. Nino se blottit contre le manteau. Merci, Nino. Le manteau sent la pluie, un peu tiède. Il est chaud. Nino pose la joue sur le manteau. Ça sent la pluie. La capuche est mouillée, Nino ? Un peu. Tu vois le point, Nino ? Oui, papa. Le bateau tient, un peu déchiré. On le garde. Une goutte passe sur la capuche. Elle tape. On reste ici, Nino ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1816,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1848,28 +1905,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de capuche</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1878,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1892,18 +1953,51 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=papier_se_dechire_bateau_part_il_refuse_de_foncer; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino sèche ses joues.
-narrateur|Le parc sent encore le bois mouillé.
-maman|On rentre quand tu es prêt ?
-enfant-m|Encore le banc.
-papa|On reste. Tu as bien demandé le câlin.
-enfant-m|Je suis moins triste.
-maman|Le câlin est encore là.
-narrateur|Ils restent au banc, tout près.
-narrateur|La flaque ne bouge plus.</t>
+          <t>narrateur|Maman pousse un peu l'herbe près de l'eau.
+narrateur|L'herbe est un peu froide.
+enfant-m|Le bateau, maintenant !
+narrateur|Nino approche la main, trop vite.
+narrateur|Le papier se déchire, plus loin.
+enfant-m|Il se déchire !
+narrateur|Le bateau part vers le milieu.
+enfant-m|Il part !
+narrateur|Nino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe la flaque, un instant.
+narrateur|Il écoute le parc, près de l'allée.
+narrateur|Sur le tissu, un éclat de capuche luit.
+enfant-m|Là, sur le tissu.
+narrateur|Nino attend, les mains ouvertes.
+enfant-m|Je veux un câlin.
+maman|Tu viens, Nino ?
+enfant-m|Oui, maman.
+narrateur|Maman ouvre les bras.
+narrateur|Nino se blottit contre le manteau.
+papa|Merci, Nino.
+narrateur|Le manteau sent la pluie, un peu tiède.
+enfant-m|Il est chaud.
+narrateur|Nino pose la joue sur le manteau.
+enfant-m|Ça sent la pluie.
+maman|La capuche est mouillée, Nino ?
+enfant-m|Un peu.
+papa|Tu vois le point, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le bateau tient, un peu déchiré.
+enfant-m|On le garde.
+maman|Une goutte passe sur la capuche.
+enfant-m|Elle tape.
+papa|On reste ici, Nino ?
+enfant-m|Oui.</t>
         </is>
       </c>
     </row>
@@ -1930,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Nino.</t>
+          <t>Ils restent près de la flaque. Maman essuie une larme sur la joue. Le bateau est parti, papa. Tu l'as vu, toi ? Oui, près de l'eau. On est bien, ici. Nino tapote le tissu du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Nino pose sa capuche contre maman. Elle est mouillée. Le bateau est resté, Nino. Oui, un peu déchiré. Ça sent la terre, un peu mouillée. Et le papier, maman. Oui, dans l'air. La goutte tape, Nino ? Oui, papa. Le bateau reste près de l'allée. Un éclat de capuche tient sur le tissu.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis triste. J'ai eu un câlin. Pleurer est permis. Bravo, Nino.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la flaque. Maman essuie une larme sur la joue. Le bateau est parti, papa. Tu l'as vu, toi ? Oui, près de l'eau. On est bien, ici. Nino tapote le tissu du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Nino pose sa capuche contre maman. Elle est mouillée. Le bateau est resté, Nino. Oui, un peu déchiré. Ça sent la terre, un peu mouillée. Et le papier, maman. Oui, dans l'air. La goutte tape, Nino ? Oui, papa. Le bateau reste près de l'allée. Un &lt;emphasis level="moderate"&gt;éclat de capuche&lt;/emphasis&gt; tient sur le tissu.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la flaque. Maman essuie une larme sur la joue. Le bateau est parti, papa. Tu l'as vu, toi ? Oui, près de l'eau. On est bien, ici. Nino tapote le tissu du doigt. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Nino pose sa capuche contre maman. Elle est mouillée. Le bateau est resté, Nino. Oui, un peu déchiré. Ça sent la terre, un peu mouillée. Et le papier, maman. Oui, dans l'air. La goutte tape, Nino ? Oui, papa. Le bateau reste près de l'allée. Un &lt;emphasis&gt;éclat de capuche&lt;/emphasis&gt; tient sur le tissu.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1987,7 +2081,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -1995,10 +2089,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2007,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2021,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de capuche</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2040,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2053,27 +2151,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_tissu; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|J'ai dit : je suis triste.
-enfant-m|J'ai eu un câlin.
-maman|Pleurer est permis.
-papa|Bravo, Nino.</t>
+          <t>narrateur|Ils restent près de la flaque.
+narrateur|Maman essuie une larme sur la joue.
+enfant-m|Le bateau est parti, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de l'eau.
+maman|On est bien, ici.
+narrateur|Nino tapote le tissu du doigt.
+enfant-m|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+narrateur|Nino pose sa capuche contre maman.
+enfant-m|Elle est mouillée.
+papa|Le bateau est resté, Nino.
+enfant-m|Oui, un peu déchiré.
+narrateur|Ça sent la terre, un peu mouillée.
+enfant-m|Et le papier, maman.
+maman|Oui, dans l'air.
+papa|La goutte tape, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le bateau reste près de l'allée.
+narrateur|Un éclat de capuche tient sur le tissu.</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2158,6 +2277,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>